<commit_message>
Renforce courriers, fournisseurs et première connexion utilisateur.
Impose le changement de mot de passe à la première connexion, sécurise les scans fournisseur/prestataire, corrige les autorisations courrier et le plafond chèque/OV, et améliore la liste des courriers avec ouverture au clic sur la ligne.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Checklist-reprise-registre-aout.xlsx
+++ b/docs/Checklist-reprise-registre-aout.xlsx
@@ -24,13 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
-  <si>
-    <t>COSUD — Checklist reprise registre d’arrivée août (209 courriers)</t>
-  </si>
-  <si>
-    <t>Une ligne = un courrier du registre papier d’août. Cocher « Statut COSUD » au fil de la saisie.</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="190">
   <si>
     <t>N° registre</t>
   </si>
@@ -53,51 +47,482 @@
     <t>Téléphone</t>
   </si>
   <si>
+    <t>Payé ?</t>
+  </si>
+  <si>
+    <t>Scan OK</t>
+  </si>
+  <si>
+    <t>Secrétaire</t>
+  </si>
+  <si>
+    <t>Statut COSUD</t>
+  </si>
+  <si>
+    <t>Bloquant</t>
+  </si>
+  <si>
+    <t>1003/DG</t>
+  </si>
+  <si>
+    <t>facture</t>
+  </si>
+  <si>
+    <t>EDITION LES SOZO</t>
+  </si>
+  <si>
+    <t>Facture N°0188, relative à la location de la hyundai Starex comptant pour le mois de juillet 2026</t>
+  </si>
+  <si>
+    <t>050333232 / 044323232</t>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>? saisir</t>
+  </si>
+  <si>
+    <t>1004/DG</t>
+  </si>
+  <si>
+    <t>BILLY SERVICES</t>
+  </si>
+  <si>
+    <t>Facture N°89/07/BS/2026, relative à la location du mini bus hyudai grand starex 775UA4</t>
+  </si>
+  <si>
+    <t>066856266 / 053999921</t>
+  </si>
+  <si>
+    <t>1006/DG</t>
+  </si>
+  <si>
+    <t>BUROTEC</t>
+  </si>
+  <si>
+    <t>Facture proforma N°S98805, relative à l'acquisition des fauteuil president chat-mix cuir noir</t>
+  </si>
+  <si>
+    <t>1008/DG</t>
+  </si>
+  <si>
+    <t>SOFT RENOVATIONS</t>
+  </si>
+  <si>
+    <t>Facture N°0058/SFTRN-ACSI/IMMO/026, relative au reglèment du mois d'Aout 2026</t>
+  </si>
+  <si>
+    <t>1009/DG</t>
+  </si>
+  <si>
+    <t>Facture N°0057/SFTRN-ACSI/IMMO/026, relative au reglèment du mois d'Aout 2026</t>
+  </si>
+  <si>
+    <t>1010/DG</t>
+  </si>
+  <si>
+    <t>SILICON CONNECT</t>
+  </si>
+  <si>
+    <t>Facture N° FAC20260701-3PFXY-SPAPW</t>
+  </si>
+  <si>
+    <t>1028/DG</t>
+  </si>
+  <si>
+    <t>ETS ND SERVICES</t>
+  </si>
+  <si>
+    <t>Proforma N°83/ENDS, relative à l'acquisition des consommables informatique</t>
+  </si>
+  <si>
+    <t>1029/DG</t>
+  </si>
+  <si>
+    <t>Facture proforma N°81/ENDS, relative à l'acquisition des consommables informatique</t>
+  </si>
+  <si>
+    <t>1030/DG</t>
+  </si>
+  <si>
+    <t>Pointe Noire</t>
+  </si>
+  <si>
+    <t>Devis estimatif de l'antenne départementale, relatif à la célébration de la fete du 15 aout 2026,</t>
+  </si>
+  <si>
+    <t>1037/DG</t>
+  </si>
+  <si>
+    <t>Facture proforma N°90/ENDS, relative à l'acquisition des matériels informatique</t>
+  </si>
+  <si>
+    <t>1038/DG</t>
+  </si>
+  <si>
+    <t>ETS DB</t>
+  </si>
+  <si>
+    <t>Facture proforma N°96, relative à l'acquisition D'une imprimante hp multifonction 179</t>
+  </si>
+  <si>
+    <t>1039/DG</t>
+  </si>
+  <si>
+    <t>BONNE NOUVELLE</t>
+  </si>
+  <si>
+    <t>Facture proforma N°178, relative à l'acquisition D'une imprimante hp multifonction 179.</t>
+  </si>
+  <si>
+    <t>1067/DG</t>
+  </si>
+  <si>
+    <t>DS POWER</t>
+  </si>
+  <si>
+    <t>Facture N°10185/2026 relative à la location gru, inverseur manuel, cable, achat carburant et main d'œuvre.</t>
+  </si>
+  <si>
+    <t>1071/DG</t>
+  </si>
+  <si>
+    <t>E²C</t>
+  </si>
+  <si>
+    <t>Facture N°0068-1169/1990, du DAF période de Juillet-Aout 2026.</t>
+  </si>
+  <si>
+    <t>1083/DG</t>
+  </si>
+  <si>
+    <t>GROUPE DREAMS LINK TECHNOLOGIES</t>
+  </si>
+  <si>
+    <t>Facture N°15/06/GDLT/26, relative au demontage et remontage du parois externe de la table de runion de la salle 2001 et demontage des ecrans pour installation des clés USB.</t>
+  </si>
+  <si>
+    <t>1086/DG</t>
+  </si>
+  <si>
+    <t>Facture N°15/12/GDLT/25, relative à l'aménagement garage DG (manuiserie metallique).</t>
+  </si>
+  <si>
+    <t>1088/DG</t>
+  </si>
+  <si>
+    <t>Facture N°16/12/GDLT/25, relative à l'aménagement garage DG, espace de repos à la Direction Générale (carrelage, pergola, peinture, grilles, serrure).</t>
+  </si>
+  <si>
+    <t>1090/DG</t>
+  </si>
+  <si>
+    <t>Facture N°021/12/GDLT/25, relative aux travaux d'amenagement du bureau du DDSAIT à la Direction Générale,</t>
+  </si>
+  <si>
+    <t>1092/DG</t>
+  </si>
+  <si>
+    <t>Facture N°22/12/GDLT/25, relative à l'amenageùent des bureaux de la DDSAIT (Fourniture et pose des portes, pose d'une loquette, plafond et plomberie,</t>
+  </si>
+  <si>
+    <t>1094/DG</t>
+  </si>
+  <si>
+    <t>Facture N°19/12/GDLT/25, relative à l'amenagement de la salle de réunion (pose d'une moquette, revision du circuit électrique et nettoyage clim).</t>
+  </si>
+  <si>
+    <t>1096/DG</t>
+  </si>
+  <si>
+    <t>Facture N°20/12/GDLT/25, relative à l'amenagement de la salle de reunion (Fourniture et pose des stores jours et nuit, plafond acoustique, panneau mural, fenetre et porte et choix et fourniture de bureau).</t>
+  </si>
+  <si>
+    <t>1098/DG</t>
+  </si>
+  <si>
+    <t>Facture N°14/12/GDLT/25, relative aux travaux de peinture, de carrelage et de deplacement du circuit de climatisation bureaux de la DSTF à la Direction Générale.</t>
+  </si>
+  <si>
+    <t>1100/DG</t>
+  </si>
+  <si>
+    <t>Facture N°15/12/GDLT/25, relative aux travaux de pose de baies vitree et cloison de separation des bureaux de la DSTF à la Direction Générale</t>
+  </si>
+  <si>
+    <t>1102/DG</t>
+  </si>
+  <si>
+    <t>Facture N°16/12/GDLT/25, relative à la fourniture et pose d'un plafond et choix, fourniture et installation des portes en bois de la DSTF à la Direction Générale.</t>
+  </si>
+  <si>
+    <t>1104/DG</t>
+  </si>
+  <si>
+    <t>Facture N°17/12/GDLT/25, relative aux travaux de fourniture et pose de panneau mural, moquette et de plomberie ainsi que d'électricité des bureaux de la DSTF à la Direction Générale.</t>
+  </si>
+  <si>
+    <t>1106/DG</t>
+  </si>
+  <si>
+    <t>Facture N°18/12/GDLT/25, relative à l'2tancheité, fourniture et pose des stores jours et nuits et d'une moquette dans les bureaux de la Direction Générale.</t>
+  </si>
+  <si>
+    <t>1109/DG</t>
+  </si>
+  <si>
+    <t>Facture N°20/12/GDLT/25, relative à l'amenagement des bureaux de la DCCC.</t>
+  </si>
+  <si>
+    <t>1111/DG</t>
+  </si>
+  <si>
+    <t>Facture N°30/12/GDLT/25, relative à l'aménagement des bureaux de la Direction du Contrôleur de Gestion à la Direction Générale.</t>
+  </si>
+  <si>
+    <t>1113/DG</t>
+  </si>
+  <si>
+    <t>Facture N°28/12/GDLT/25, relative à la facilitation de la circulation dans la cour de l'Agence à la Direction Générale en période de pluie (Renforcement de la dalle de la cour, renforcement de la structure enfuit, mener et repli du matériels).</t>
+  </si>
+  <si>
+    <t>1115/DG</t>
+  </si>
+  <si>
+    <t>Facture N°24/12/GDLT/25, relative à l'aménagement des bureaux de la DISSI</t>
+  </si>
+  <si>
+    <t>1117/DG</t>
+  </si>
+  <si>
+    <t>Facture N°34/12/GDLT/25, relative à l'aménagement des conteneurs</t>
+  </si>
+  <si>
+    <t>1119/DG</t>
+  </si>
+  <si>
+    <t>Facture N°47/08/GDLT/25, relative à l'aménagement des bureaux de la DISI (application peinture et installation des stores).</t>
+  </si>
+  <si>
+    <t>1121/DG</t>
+  </si>
+  <si>
+    <t>Facture N°48/08/GDLT/25, relative à l'aménagement des bureaux de madame la DISI (electricité, déplacement circuit climatisation, fourniture et pose d'un plafond acoustique)</t>
+  </si>
+  <si>
+    <t>1123/DG</t>
+  </si>
+  <si>
+    <t>Facture N°49/08/GDLT/25, relative à l'aménagement des bureaux de la DISI (carrelage, plomberie, fourniture et pose d'une moquette).</t>
+  </si>
+  <si>
+    <t>1125DG</t>
+  </si>
+  <si>
+    <t>Facture N°50/08/GDLT/25, relative à l'amenagement des bureaux de madame la DISI (fabrication et pose des cloisons de separation et de micro perfores).</t>
+  </si>
+  <si>
+    <t>1126/DG</t>
+  </si>
+  <si>
+    <t>Facture proforma N°10180/2026, inverseur manuel, cable, achat carburant, main d'œuvre manutention, location groupe 44KVA (2mois)</t>
+  </si>
+  <si>
+    <t>1127/DG</t>
+  </si>
+  <si>
+    <t>Devis N°10179/2026, relative à</t>
+  </si>
+  <si>
+    <t>1128/DG</t>
+  </si>
+  <si>
+    <t>LCDE</t>
+  </si>
+  <si>
+    <t>Paiement Facture LCDE de la Direction Générale mois Aout 2026,</t>
+  </si>
+  <si>
+    <t>1130/DG</t>
+  </si>
+  <si>
+    <t>ETS DALPIVOT AIR FROID</t>
+  </si>
+  <si>
+    <t>Facture N°01, relative à la prestation de maintenance préventive du mois de janvier 2026</t>
+  </si>
+  <si>
+    <t>1131/DG</t>
+  </si>
+  <si>
+    <t>Facture N°02, relative à la prestation de maintenance préventive du mois de Févrie 2026</t>
+  </si>
+  <si>
+    <t>1132/DG</t>
+  </si>
+  <si>
+    <t>Facture N°03, relative à la prestation de maintenance préventive du mois de Mars 2026</t>
+  </si>
+  <si>
+    <t>1133/DG</t>
+  </si>
+  <si>
+    <t>Facture N°04, relative à la prestation de maintenance préventive du mois de Avril 2026</t>
+  </si>
+  <si>
+    <t>1134/DG</t>
+  </si>
+  <si>
+    <t>Facture N°05, relative à la prestation de maintenance préventive du mois de Mai 2026</t>
+  </si>
+  <si>
+    <t>1135/DG</t>
+  </si>
+  <si>
+    <t>Facture N°06, relative à la prestation de maintenance préventive du mois de Juin 2026</t>
+  </si>
+  <si>
+    <t>1136/DG</t>
+  </si>
+  <si>
+    <t>Facture N°07, relative à la prestation de maintenance préventive du mois de Juillet 2026</t>
+  </si>
+  <si>
+    <t>1145/DG</t>
+  </si>
+  <si>
+    <t>Facture N° 0189, relative à la location de la hyundai grand starex comptant pour le mois d'aout 2026</t>
+  </si>
+  <si>
+    <t>1150/DG</t>
+  </si>
+  <si>
+    <t>CONGO TELECOM</t>
+  </si>
+  <si>
+    <t>Facture N°F26080907948CT, relative au paiement postpayé speed pro 100 site bureau DG
+IP Adress SITE BUREAU DG
+Speed-Business-Bronze site ACSI</t>
+  </si>
+  <si>
+    <t>1151/DG</t>
+  </si>
+  <si>
+    <t>KUDIA</t>
+  </si>
+  <si>
+    <t>Facture N°124/09/KU/26, relative au paiement de la prestation de restauration et livraison des plats de la cantine, pour 32 personnes facturées au prix de 7250/personne sur 26 jours/Mois</t>
+  </si>
+  <si>
+    <t>1152/DG</t>
+  </si>
+  <si>
+    <t>AFRIQUE AUTOMOBILE</t>
+  </si>
+  <si>
+    <t>Facture N°9503, relative à l'acquisition d'un pneus pour la 032GGQ4,</t>
+  </si>
+  <si>
+    <t>1154/DG</t>
+  </si>
+  <si>
+    <t>AUTO MOBILE TOYOTA D'ORIGINE PIECES</t>
+  </si>
+  <si>
+    <t>Facture Proforma N°003031, relative à l'acquisition d'un pneus pour la 032GGQ4,</t>
+  </si>
+  <si>
+    <t>1157/DG</t>
+  </si>
+  <si>
+    <t>Devis N°S113104, relative à l'acquisition d'une television TCL 98 LED SMART 4K</t>
+  </si>
+  <si>
+    <t>1160/DG</t>
+  </si>
+  <si>
+    <t>Facture N°125/KUDIA/09/26, relative au paiement de la prestation de restauration et livraison des plats de la cantine, pour 18 personnes facturées au prix de 7250/personne sur 26 jours/Mois, site virage Maya-Maya</t>
+  </si>
+  <si>
+    <t>1170/DG</t>
+  </si>
+  <si>
+    <t>PUMA</t>
+  </si>
+  <si>
+    <t>Proforma relative à la vidange de la 032GGQ4</t>
+  </si>
+  <si>
+    <t>1174/DG</t>
+  </si>
+  <si>
+    <t>METRE DE LUXE</t>
+  </si>
+  <si>
+    <t>Facture N°0051, relative au paiement du mois de Septembre 2026</t>
+  </si>
+  <si>
+    <t>1177/DG</t>
+  </si>
+  <si>
+    <t>PHARMACIE MAVRE</t>
+  </si>
+  <si>
+    <t>Justificatif de solde tiers</t>
+  </si>
+  <si>
+    <t>1181/DG</t>
+  </si>
+  <si>
+    <t>Proforma N°158 relative à la vidange de la 901 GDQ4</t>
+  </si>
+  <si>
+    <t>1182/DG</t>
+  </si>
+  <si>
+    <t>1190/DG</t>
+  </si>
+  <si>
+    <t>AF,COM</t>
+  </si>
+  <si>
+    <t>Facture N°174/09/AFCOM/2026, relative au paiement du mois de septembre 2026</t>
+  </si>
+  <si>
+    <t>Utilité des colonnes (programme reprise §8)</t>
+  </si>
+  <si>
+    <t>Colonne</t>
+  </si>
+  <si>
+    <t>Utilité</t>
+  </si>
+  <si>
+    <t>Identifiant papier / COSUD</t>
+  </si>
+  <si>
+    <t>Contrôle</t>
+  </si>
+  <si>
+    <t>facture / MAD / autre</t>
+  </si>
+  <si>
+    <t>Libellé</t>
+  </si>
+  <si>
+    <t>Résumé</t>
+  </si>
+  <si>
+    <t>Obligatoire si facture</t>
+  </si>
+  <si>
+    <t>Obligatoire facture / demande (SMS)</t>
+  </si>
+  <si>
     <t>Payé ? / Reliquat ?</t>
   </si>
   <si>
-    <t>Scan OK</t>
-  </si>
-  <si>
-    <t>Secrétaire</t>
-  </si>
-  <si>
-    <t>Statut COSUD</t>
-  </si>
-  <si>
-    <t>Bloquant</t>
-  </si>
-  <si>
-    <t>Utilité des colonnes (programme reprise §8)</t>
-  </si>
-  <si>
-    <t>Colonne</t>
-  </si>
-  <si>
-    <t>Utilité</t>
-  </si>
-  <si>
-    <t>Identifiant papier / COSUD</t>
-  </si>
-  <si>
-    <t>Contrôle</t>
-  </si>
-  <si>
-    <t>facture / MAD / autre</t>
-  </si>
-  <si>
-    <t>Libellé</t>
-  </si>
-  <si>
-    <t>Résumé</t>
-  </si>
-  <si>
-    <t>Obligatoire si facture</t>
-  </si>
-  <si>
-    <t>Obligatoire facture / demande (SMS)</t>
-  </si>
-  <si>
     <t>Aide dettes après saisie</t>
   </si>
   <si>
@@ -168,13 +593,16 @@
   </si>
   <si>
     <t>~69 + contrôle</t>
+  </si>
+  <si>
+    <t>à saisir</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -210,8 +638,12 @@
       <color rgb="FF06A269"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -233,8 +665,13 @@
         <fgColor rgb="FFE8F8F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9FAFB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -257,11 +694,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -277,6 +729,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -586,900 +1063,1940 @@
   <dimension ref="A1:L213"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="36" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="1" max="1" width="16" style="9" customWidth="1"/>
+    <col min="2" max="2" width="14" style="9" customWidth="1"/>
+    <col min="3" max="3" width="12" style="9" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" style="9" customWidth="1"/>
+    <col min="5" max="5" width="36" style="9" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="8.77734375" style="9" customWidth="1"/>
+    <col min="8" max="9" width="8.21875" style="9" customWidth="1"/>
+    <col min="10" max="10" width="9.88671875" style="9" customWidth="1"/>
+    <col min="11" max="11" width="14" style="9" customWidth="1"/>
+    <col min="12" max="12" width="28" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18">
-      <c r="A1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
+    <row r="1" spans="1:12" ht="18" customHeight="1">
+      <c r="A1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
     </row>
     <row r="4" spans="1:12" ht="28.05" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:12" ht="41.4">
+      <c r="A5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
+      <c r="B5" s="11">
+        <v>46237</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="12">
+        <v>3120000</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="10"/>
+    </row>
+    <row r="6" spans="1:12" ht="41.4">
+      <c r="A6" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="15">
+        <v>46237</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="16">
+        <v>3120000</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="14"/>
+    </row>
+    <row r="7" spans="1:12" ht="28.8" customHeight="1">
+      <c r="A7" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="11">
+        <v>46237</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="12">
+        <v>1292567</v>
+      </c>
+      <c r="G7" s="13"/>
+      <c r="H7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L7" s="10"/>
+    </row>
+    <row r="8" spans="1:12" ht="27.6">
+      <c r="A8" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="15">
+        <v>46238</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="16">
+        <v>1800000</v>
+      </c>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L8" s="14"/>
+    </row>
+    <row r="9" spans="1:12" ht="27.6">
+      <c r="A9" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="11">
+        <v>46238</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="12">
+        <v>1500000</v>
+      </c>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L9" s="10"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-    </row>
-    <row r="16" spans="1:12">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="1:12">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-    </row>
-    <row r="20" spans="1:12">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-    </row>
-    <row r="21" spans="1:12">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-    </row>
-    <row r="22" spans="1:12">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="1:12">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-    </row>
-    <row r="24" spans="1:12">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="1:12">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-    </row>
-    <row r="27" spans="1:12">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-    </row>
-    <row r="28" spans="1:12">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-    </row>
-    <row r="29" spans="1:12">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="1:12">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
-    </row>
-    <row r="31" spans="1:12">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-    </row>
-    <row r="32" spans="1:12">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="3"/>
-    </row>
-    <row r="33" spans="1:12">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-    </row>
-    <row r="34" spans="1:12">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="3"/>
-    </row>
-    <row r="35" spans="1:12">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-    </row>
-    <row r="36" spans="1:12">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="3"/>
-    </row>
-    <row r="37" spans="1:12">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-    </row>
-    <row r="38" spans="1:12">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
-    </row>
-    <row r="39" spans="1:12">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-    </row>
-    <row r="40" spans="1:12">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
-      <c r="K40" s="3"/>
-      <c r="L40" s="3"/>
+      <c r="A10" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="15">
+        <v>46239</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="16">
+        <v>1550047</v>
+      </c>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="L10" s="14"/>
+    </row>
+    <row r="11" spans="1:12" ht="27.6">
+      <c r="A11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="11">
+        <v>46244</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="12">
+        <v>3715625</v>
+      </c>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L11" s="10"/>
+    </row>
+    <row r="12" spans="1:12" ht="41.4">
+      <c r="A12" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="15">
+        <v>46244</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="16">
+        <v>832300</v>
+      </c>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="14"/>
+    </row>
+    <row r="13" spans="1:12" ht="41.4">
+      <c r="A13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="11">
+        <v>46244</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="12">
+        <v>1500000</v>
+      </c>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L13" s="10"/>
+    </row>
+    <row r="14" spans="1:12" ht="27.6">
+      <c r="A14" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="15">
+        <v>46244</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="16">
+        <v>588555</v>
+      </c>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L14" s="14"/>
+    </row>
+    <row r="15" spans="1:12" ht="41.4">
+      <c r="A15" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="11">
+        <v>46244</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="12">
+        <v>624225</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" s="10"/>
+    </row>
+    <row r="16" spans="1:12" ht="41.4">
+      <c r="A16" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="15">
+        <v>46244</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="16">
+        <v>606390</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" s="14"/>
+    </row>
+    <row r="17" spans="1:12" ht="41.4">
+      <c r="A17" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="11">
+        <v>46247</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="12">
+        <v>725000</v>
+      </c>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" s="10"/>
+    </row>
+    <row r="18" spans="1:12" ht="27.6">
+      <c r="A18" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="15">
+        <v>46247</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" s="16">
+        <v>51289</v>
+      </c>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L18" s="14"/>
+    </row>
+    <row r="19" spans="1:12" ht="69">
+      <c r="A19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F19" s="12">
+        <v>202130</v>
+      </c>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L19" s="10"/>
+    </row>
+    <row r="20" spans="1:12" ht="41.4">
+      <c r="A20" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="16">
+        <v>5756543</v>
+      </c>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L20" s="14"/>
+    </row>
+    <row r="21" spans="1:12" ht="55.2">
+      <c r="A21" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F21" s="12">
+        <v>6182800</v>
+      </c>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L21" s="10"/>
+    </row>
+    <row r="22" spans="1:12" ht="41.4">
+      <c r="A22" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="16">
+        <v>7499618</v>
+      </c>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L22" s="14"/>
+    </row>
+    <row r="23" spans="1:12" ht="55.2">
+      <c r="A23" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="12">
+        <v>7303433</v>
+      </c>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L23" s="10"/>
+    </row>
+    <row r="24" spans="1:12" ht="55.2">
+      <c r="A24" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" s="16">
+        <v>6836750</v>
+      </c>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L24" s="14"/>
+    </row>
+    <row r="25" spans="1:12" ht="69">
+      <c r="A25" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="12">
+        <v>5826100</v>
+      </c>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L25" s="10"/>
+    </row>
+    <row r="26" spans="1:12" ht="55.2">
+      <c r="A26" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F26" s="16">
+        <v>8294342</v>
+      </c>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J26" s="14"/>
+      <c r="K26" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L26" s="14"/>
+    </row>
+    <row r="27" spans="1:12" ht="55.2">
+      <c r="A27" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="12">
+        <v>9018684</v>
+      </c>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L27" s="10"/>
+    </row>
+    <row r="28" spans="1:12" ht="55.2">
+      <c r="A28" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F28" s="16">
+        <v>9274200</v>
+      </c>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L28" s="14"/>
+    </row>
+    <row r="29" spans="1:12" ht="69">
+      <c r="A29" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" s="12">
+        <v>7342075</v>
+      </c>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L29" s="10"/>
+    </row>
+    <row r="30" spans="1:12" ht="55.2">
+      <c r="A30" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="F30" s="16">
+        <v>8458689</v>
+      </c>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L30" s="14"/>
+    </row>
+    <row r="31" spans="1:12" ht="27.6">
+      <c r="A31" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B31" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F31" s="12">
+        <v>6553200</v>
+      </c>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L31" s="10"/>
+    </row>
+    <row r="32" spans="1:12" ht="55.2">
+      <c r="A32" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B32" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F32" s="16">
+        <v>6669291</v>
+      </c>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L32" s="14"/>
+    </row>
+    <row r="33" spans="1:12" ht="82.8">
+      <c r="A33" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F33" s="12">
+        <v>8615494</v>
+      </c>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L33" s="10"/>
+    </row>
+    <row r="34" spans="1:12" ht="27.6">
+      <c r="A34" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="F34" s="16">
+        <v>9861566</v>
+      </c>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L34" s="14"/>
+    </row>
+    <row r="35" spans="1:12" ht="27.6">
+      <c r="A35" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B35" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="F35" s="12">
+        <v>4253647</v>
+      </c>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L35" s="10"/>
+    </row>
+    <row r="36" spans="1:12" ht="55.2">
+      <c r="A36" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F36" s="16">
+        <v>7728500</v>
+      </c>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L36" s="14"/>
+    </row>
+    <row r="37" spans="1:12" ht="69">
+      <c r="A37" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F37" s="12">
+        <v>9422825</v>
+      </c>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L37" s="10"/>
+    </row>
+    <row r="38" spans="1:12" ht="55.2">
+      <c r="A38" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="15">
+        <v>46248</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F38" s="16">
+        <v>8251660</v>
+      </c>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J38" s="14"/>
+      <c r="K38" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L38" s="14"/>
+    </row>
+    <row r="39" spans="1:12" ht="55.2">
+      <c r="A39" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B39" s="11">
+        <v>46248</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F39" s="12">
+        <v>3749395</v>
+      </c>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="1:12" ht="55.2">
+      <c r="A40" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="15">
+        <v>46253</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="F40" s="16">
+        <v>2306660</v>
+      </c>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J40" s="14"/>
+      <c r="K40" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L40" s="14"/>
     </row>
     <row r="41" spans="1:12">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-    </row>
-    <row r="42" spans="1:12">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-    </row>
-    <row r="43" spans="1:12">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="2"/>
-      <c r="I43" s="2"/>
-      <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-    </row>
-    <row r="44" spans="1:12">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
-      <c r="K44" s="3"/>
-      <c r="L44" s="3"/>
-    </row>
-    <row r="45" spans="1:12">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-    </row>
-    <row r="46" spans="1:12">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="J46" s="3"/>
-      <c r="K46" s="3"/>
-      <c r="L46" s="3"/>
-    </row>
-    <row r="47" spans="1:12">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-    </row>
-    <row r="48" spans="1:12">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
-      <c r="J48" s="3"/>
-      <c r="K48" s="3"/>
-      <c r="L48" s="3"/>
-    </row>
-    <row r="49" spans="1:12">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
-      <c r="I49" s="2"/>
-      <c r="J49" s="2"/>
-      <c r="K49" s="2"/>
-      <c r="L49" s="2"/>
-    </row>
-    <row r="50" spans="1:12">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="3"/>
-      <c r="K50" s="3"/>
-      <c r="L50" s="3"/>
-    </row>
-    <row r="51" spans="1:12">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
-      <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-    </row>
-    <row r="52" spans="1:12">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
-      <c r="I52" s="3"/>
-      <c r="J52" s="3"/>
-      <c r="K52" s="3"/>
-      <c r="L52" s="3"/>
-    </row>
-    <row r="53" spans="1:12">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-    </row>
-    <row r="54" spans="1:12">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="J54" s="3"/>
-      <c r="K54" s="3"/>
-      <c r="L54" s="3"/>
-    </row>
-    <row r="55" spans="1:12">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
-      <c r="L55" s="2"/>
-    </row>
-    <row r="56" spans="1:12">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="3"/>
-      <c r="I56" s="3"/>
-      <c r="J56" s="3"/>
-      <c r="K56" s="3"/>
-      <c r="L56" s="3"/>
-    </row>
-    <row r="57" spans="1:12">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
-      <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-    </row>
-    <row r="58" spans="1:12">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3"/>
-      <c r="I58" s="3"/>
-      <c r="J58" s="3"/>
-      <c r="K58" s="3"/>
-      <c r="L58" s="3"/>
+      <c r="A41" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" s="11">
+        <v>46253</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="F41" s="12">
+        <v>8944000</v>
+      </c>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="1:12" ht="27.6">
+      <c r="A42" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="15">
+        <v>46253</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="E42" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="F42" s="16">
+        <v>55824</v>
+      </c>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L42" s="14"/>
+    </row>
+    <row r="43" spans="1:12" ht="41.4">
+      <c r="A43" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" s="11">
+        <v>46253</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F43" s="12">
+        <v>340000</v>
+      </c>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L43" s="10"/>
+    </row>
+    <row r="44" spans="1:12" ht="41.4">
+      <c r="A44" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B44" s="15">
+        <v>46253</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="16">
+        <v>340000</v>
+      </c>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I44" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J44" s="14"/>
+      <c r="K44" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L44" s="14"/>
+    </row>
+    <row r="45" spans="1:12" ht="41.4">
+      <c r="A45" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B45" s="11">
+        <v>46253</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F45" s="12">
+        <v>340000</v>
+      </c>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I45" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L45" s="10"/>
+    </row>
+    <row r="46" spans="1:12" ht="41.4">
+      <c r="A46" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="B46" s="15">
+        <v>46253</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F46" s="16">
+        <v>340000</v>
+      </c>
+      <c r="G46" s="14"/>
+      <c r="H46" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L46" s="14"/>
+    </row>
+    <row r="47" spans="1:12" ht="41.4">
+      <c r="A47" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B47" s="11">
+        <v>46253</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F47" s="12">
+        <v>340000</v>
+      </c>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J47" s="10"/>
+      <c r="K47" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L47" s="10"/>
+    </row>
+    <row r="48" spans="1:12" ht="41.4">
+      <c r="A48" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B48" s="15">
+        <v>46253</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F48" s="16">
+        <v>340000</v>
+      </c>
+      <c r="G48" s="14"/>
+      <c r="H48" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I48" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J48" s="14"/>
+      <c r="K48" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L48" s="14"/>
+    </row>
+    <row r="49" spans="1:12" ht="41.4">
+      <c r="A49" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B49" s="11">
+        <v>46253</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F49" s="12">
+        <v>340000</v>
+      </c>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L49" s="10"/>
+    </row>
+    <row r="50" spans="1:12" ht="41.4">
+      <c r="A50" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="B50" s="15">
+        <v>46255</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="F50" s="16">
+        <v>3120000</v>
+      </c>
+      <c r="G50" s="14"/>
+      <c r="H50" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I50" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J50" s="14"/>
+      <c r="K50" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L50" s="14"/>
+    </row>
+    <row r="51" spans="1:12" ht="69">
+      <c r="A51" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B51" s="11">
+        <v>46255</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F51" s="12">
+        <v>1035000</v>
+      </c>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I51" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L51" s="10"/>
+    </row>
+    <row r="52" spans="1:12" ht="69">
+      <c r="A52" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B52" s="15">
+        <v>46258</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F52" s="16">
+        <v>6032000</v>
+      </c>
+      <c r="G52" s="14"/>
+      <c r="H52" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I52" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J52" s="14"/>
+      <c r="K52" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L52" s="14"/>
+    </row>
+    <row r="53" spans="1:12" ht="27.6">
+      <c r="A53" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="B53" s="11">
+        <v>46258</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="F53" s="12">
+        <v>75000</v>
+      </c>
+      <c r="G53" s="10"/>
+      <c r="H53" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J53" s="10"/>
+      <c r="K53" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L53" s="10"/>
+    </row>
+    <row r="54" spans="1:12" ht="27.6">
+      <c r="A54" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B54" s="15">
+        <v>46258</v>
+      </c>
+      <c r="C54" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="F54" s="16">
+        <v>85000</v>
+      </c>
+      <c r="G54" s="14"/>
+      <c r="H54" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I54" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J54" s="14"/>
+      <c r="K54" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L54" s="14"/>
+    </row>
+    <row r="55" spans="1:12" ht="27.6">
+      <c r="A55" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B55" s="11">
+        <v>46258</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F55" s="12">
+        <v>3565811</v>
+      </c>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J55" s="10"/>
+      <c r="K55" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L55" s="10"/>
+    </row>
+    <row r="56" spans="1:12" ht="82.8">
+      <c r="A56" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B56" s="15">
+        <v>46258</v>
+      </c>
+      <c r="C56" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F56" s="16">
+        <v>3393000</v>
+      </c>
+      <c r="G56" s="14"/>
+      <c r="H56" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I56" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J56" s="14"/>
+      <c r="K56" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L56" s="14"/>
+    </row>
+    <row r="57" spans="1:12" ht="27.6">
+      <c r="A57" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B57" s="11">
+        <v>46258</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="F57" s="12">
+        <v>70000</v>
+      </c>
+      <c r="G57" s="10"/>
+      <c r="H57" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J57" s="10"/>
+      <c r="K57" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L57" s="10"/>
+    </row>
+    <row r="58" spans="1:12" ht="27.6">
+      <c r="A58" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="B58" s="15">
+        <v>46258</v>
+      </c>
+      <c r="C58" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E58" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="F58" s="16">
+        <v>649294</v>
+      </c>
+      <c r="G58" s="14"/>
+      <c r="H58" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I58" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J58" s="14"/>
+      <c r="K58" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L58" s="14"/>
     </row>
     <row r="59" spans="1:12">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
-      <c r="I59" s="2"/>
-      <c r="J59" s="2"/>
-      <c r="K59" s="2"/>
-      <c r="L59" s="2"/>
-    </row>
-    <row r="60" spans="1:12">
-      <c r="A60" s="3"/>
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
-      <c r="G60" s="3"/>
-      <c r="H60" s="3"/>
-      <c r="I60" s="3"/>
-      <c r="J60" s="3"/>
-      <c r="K60" s="3"/>
-      <c r="L60" s="3"/>
-    </row>
-    <row r="61" spans="1:12">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
-      <c r="I61" s="2"/>
-      <c r="J61" s="2"/>
-      <c r="K61" s="2"/>
-      <c r="L61" s="2"/>
-    </row>
-    <row r="62" spans="1:12">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
-      <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3"/>
-      <c r="I62" s="3"/>
-      <c r="J62" s="3"/>
-      <c r="K62" s="3"/>
-      <c r="L62" s="3"/>
+      <c r="A59" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B59" s="11">
+        <v>46258</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F59" s="12">
+        <v>1171607</v>
+      </c>
+      <c r="G59" s="10"/>
+      <c r="H59" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I59" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J59" s="10"/>
+      <c r="K59" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L59" s="10"/>
+    </row>
+    <row r="60" spans="1:12" ht="27.6">
+      <c r="A60" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="B60" s="15">
+        <v>46258</v>
+      </c>
+      <c r="C60" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="F60" s="14"/>
+      <c r="G60" s="14"/>
+      <c r="H60" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I60" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J60" s="14"/>
+      <c r="K60" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L60" s="14"/>
+    </row>
+    <row r="61" spans="1:12" ht="27.6">
+      <c r="A61" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B61" s="11">
+        <v>46258</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="F61" s="12">
+        <v>60000</v>
+      </c>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I61" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J61" s="10"/>
+      <c r="K61" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="L61" s="10"/>
+    </row>
+    <row r="62" spans="1:12" ht="27.6">
+      <c r="A62" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="B62" s="15">
+        <v>46259</v>
+      </c>
+      <c r="C62" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="E62" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="F62" s="16">
+        <v>247090</v>
+      </c>
+      <c r="G62" s="14"/>
+      <c r="H62" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="I62" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J62" s="14"/>
+      <c r="K62" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="L62" s="14"/>
     </row>
     <row r="63" spans="1:12">
       <c r="A63" s="2"/>
@@ -3624,166 +5141,166 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="48" customWidth="1"/>
+    <col min="1" max="1" width="28" style="9" customWidth="1"/>
+    <col min="2" max="2" width="48" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18">
-      <c r="A1" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="10"/>
+    <row r="1" spans="1:2" ht="18" customHeight="1">
+      <c r="A1" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="19"/>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>155</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>17</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="6" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>19</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>20</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>21</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>22</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>23</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="6" t="s">
-        <v>9</v>
+        <v>164</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>24</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>25</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>26</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>27</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.6">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.6" customHeight="1">
       <c r="A17" s="7" t="s">
-        <v>29</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="10"/>
+      <c r="A18" s="21" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="19"/>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="10"/>
+      <c r="A19" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="19"/>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="10"/>
+      <c r="A20" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="19"/>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="10"/>
+      <c r="A21" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="B21" s="19"/>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="10"/>
+      <c r="A22" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="B22" s="19"/>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="10"/>
+      <c r="A23" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="19"/>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="10"/>
+      <c r="A24" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3805,44 +5322,44 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="1" max="1" width="14" style="9" customWidth="1"/>
+    <col min="2" max="2" width="18" style="9" customWidth="1"/>
+    <col min="3" max="4" width="12" style="9" customWidth="1"/>
+    <col min="5" max="5" width="40" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18">
-      <c r="A1" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
+    <row r="1" spans="1:5" ht="18" customHeight="1">
+      <c r="A1" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="4" t="s">
-        <v>38</v>
+        <v>179</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>40</v>
+        <v>181</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>41</v>
+        <v>182</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>42</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="8" t="s">
-        <v>43</v>
+        <v>184</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -3850,10 +5367,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="8" t="s">
-        <v>45</v>
+        <v>186</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -3861,10 +5378,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="8" t="s">
-        <v>46</v>
+        <v>187</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>47</v>
+        <v>188</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>

</xml_diff>